<commit_message>
feat: TASK-005 money and time helpers, auth/rate-limit error codes, log text redaction
- Money helpers: bigint minor units (EGP piastres), exact arithmetic, one
  HALF-UP rounding implementation with ties away from zero (R9, R22).
- Time helpers: UTC instants, Clock, strict offset-required parsing, exact
  durations, Africa/Cairo calendar days with DST (R20, R21).
- Error codes UNAUTHENTICATED (401) and RATE_LIMITED (429) per API contract
  §6.1/§29.
- Logger masks secrets embedded in text (msg, error message/stack, causes).
- Record owner decisions R20-R22 in the business spec and ledger, add
  ADR-0011, align day-window wording across docs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/decisions/business-rules-ledger.xlsx
+++ b/docs/decisions/business-rules-ledger.xlsx
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Decision"/>
@@ -7392,7 +7392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="26" min="1" max="1"/>
@@ -7780,6 +7780,87 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>R20</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Business Timezone</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>The business timezone is Africa/Cairo, including daylight saving time when Egypt applies it. Timestamps are stored in UTC. Calendar-day concepts (analytics Today/Yesterday/ranges, the return window) use Africa/Cairo.</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-005). Clarifies DB Design §1 principle 10, Q17 and Q149. Business Spec R20.</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>R21</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Day Counting</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Return window: a return may be requested until the end of the 14th calendar day after the delivery date in Africa/Cairo (delivery day is day 0). COD confirmation maximum: an exact elapsed duration of at most 72 hours from order creation; the configurable timeout can never exceed 72 hours.</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-005). Clarifies Q17 and Q25. Business Spec R21.</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>R22</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>HALF-UP on Negative Amounts</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>HALF-UP rounding ties round away from zero for negative amounts too (2.5 → 3, -2.5 → -3).</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-005). Clarifies R9. Business Spec R22.</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs: TASK-007 record owner decisions R23-R27 and ADR-0013
- Business spec: R23-R27 (sessions after reset/change, login throttling,
  WhatsApp phone verification and non-reserving pending registrations,
  no login with an unverified email, Egyptian mobile numbers only).
- Ledger: R23-R27 rows in "Closure & Audit Decisions".
- ADR-0013 (amends ADR-0008): opaque tokens with rotation and reuse
  detection, cookie vs Bearer transport, Origin/Referer CSRF check,
  PostgreSQL throttling store, client IP via a thin custom server,
  scrypt parameters and the offline common-password list.
- DB design, API contract, security requirements, user flows and
  architecture updated; TASK-002/TASK-002A open items resolved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/decisions/business-rules-ledger.xlsx
+++ b/docs/decisions/business-rules-ledger.xlsx
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Decision"/>
@@ -7392,7 +7392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="26" min="1" max="1"/>
@@ -7861,6 +7861,141 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>R23</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Sessions After Password Reset / Change</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>A password reset revokes all of the customer's sessions. A password change while logged in keeps the current session and revokes all others. A customer session lasts 30 days from login; the lifetime is absolute (refreshing does not extend it).</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-007 + plan review). Completes User Flows §3.2; clarifies Q162, Q164. Resolves TASK-002A open decision 2 for customers. Business Spec R23.</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>R24</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Login Throttling</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>5 consecutive failed password attempts on an account block that account's login for 15 minutes; the correct password is also refused during the block; the count resets on a successful login and after the block; wrong current passwords during a password change count. Per IP: 30 failed logins within 15 minutes block logins from that IP for 15 minutes. CAPTCHA is added later (TASK-061).</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-007 + plan review); per-IP threshold proposed in TASK-007 (ADR-0013) and approved. Implements Q157. Business Spec R24.</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>R25</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Phone Verification &amp; Account Activation</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>At registration the phone is verified by a WhatsApp OTP and the email by an email OTP; the account becomes ACTIVE only after both. Registration requires email, phone, password and full name. WhatsApp is also the OTP channel for phone change and guest-order claim. Pending registrations do not reserve identifiers: email/phone uniqueness applies only to verified identities (Q151 applies to a verified email). A PENDING_VERIFICATION account expires 24 hours after registration. A new registration replaces a pending account whose email and phone are both unverified, or any expired pending account; a pending account with a verified email keeps it, and whichever account verifies a shared unverified phone first keeps it.</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-007 + plan review). Extends Q41, Q42, Q44, Q151, Q153. Resolves TASK-002A open decision 3. Business Spec R25.</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>R26</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Unverified Email Cannot Log In</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>A customer whose email is not verified cannot log in. A customer whose email is verified but whose phone is not yet verified (pending, within 24 hours) can log in with access limited to session actions and verification steps; everything else requires an ACTIVE account.</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-007 + plan review). Business Spec R26.</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>R27</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Customer Phone Format</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Customer phone numbers are Egyptian mobile numbers only (010, 011, 012 or 015 followed by 8 digits), stored normalized in E.164 (+20…). Accepted input forms: 01xxxxxxxxx, +201xxxxxxxxx, 00201xxxxxxxxx.</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (TASK-007 plan review). Clarifies Q41, R13. Business Spec R27.</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs: record Phase 1 staff and OTP decisions (R28–R31)
Owner decisions of 2026-10-01: email OTP for all staff with 30-day
trusted devices, 12 h / 60 min staff session defaults, staff reset
revokes all sessions, email as the only OTP channel (phone change OTP
to the verified email, amends R25), guest order claim OTP to the
order's email. Registration phone verification stays open.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015UfRXeQxrrequZWe28vACh
</commit_message>
<xml_diff>
--- a/docs/decisions/business-rules-ledger.xlsx
+++ b/docs/decisions/business-rules-ledger.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BeautyFits Q1-Q185" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closure C1-C6" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Corrections" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closure &amp; Audit Decisions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BeautyFits Q1-Q185" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Closure C1-C6" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Audit Corrections" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Closure &amp; Audit Decisions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -7392,7 +7392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="26" min="1" max="1"/>
@@ -7996,6 +7996,114 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>R28</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Employee Second Factor</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Every employee, Owner/Admin included, logs in with email + password + email OTP. A successful OTP trusts that device for 30 days; after 30 days or on a new device the OTP is required again. No separate MFA factor in v1.</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-01, project thread). Amends Q165. Business Spec R28.</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>R29</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Staff Sessions</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Default staff session: 12 hours maximum, ended after 60 minutes without activity; both configurable by the Owner/Admin. A staff password reset revokes all of the employee's sessions (as R23 for customers).</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-01, project thread). Clarifies Q163. Business Spec R29.</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>R30</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Email as the Only OTP Channel</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Email is the only OTP channel in v1 for customers and employees (SMS/WhatsApp OTP cost more). Phone change: re-authenticate, OTP to the verified account email, change phone, notify the verified email. Email change unchanged (Q152). Registration phone verification: BUSINESS DECISION REQUIRED.</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-01, project thread). Amends Q153 and the WhatsApp channel of R25. Business Spec R30.</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>R31</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Guest Order Claim OTP</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>The claim OTP is emailed to the guest_email stored on the guest order(s). Only guest orders whose phone and email both match the account are linked; others are linked through support. Phone match alone is never sufficient.</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-01, project thread). Clarifies Q43/Q44 and User Flows §3.5; replaces the WhatsApp channel of R25. Business Spec R31.</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
docs: R30 drops the registration phone OTP (owner decision)
The account becomes ACTIVE once the email is verified; the phone stays
required, Egyptian and unique among active accounts. Amends R25/R26.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015UfRXeQxrrequZWe28vACh
</commit_message>
<xml_diff>
--- a/docs/decisions/business-rules-ledger.xlsx
+++ b/docs/decisions/business-rules-ledger.xlsx
@@ -8063,12 +8063,12 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Email is the only OTP channel in v1 for customers and employees (SMS/WhatsApp OTP cost more). Phone change: re-authenticate, OTP to the verified account email, change phone, notify the verified email. Email change unchanged (Q152). Registration phone verification: BUSINESS DECISION REQUIRED.</t>
+          <t>Email is the only OTP channel in v1 for customers and employees (SMS/WhatsApp OTP cost more). Phone change: re-authenticate, OTP to the verified account email, change phone, notify the verified email. Email change unchanged (Q152). Registration: no phone OTP; the account is ACTIVE once the email is verified; the phone stays required, Egyptian and unique among active accounts.</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Owner decision (2026-10-01, project thread). Amends Q153 and the WhatsApp channel of R25. Business Spec R30.</t>
+          <t>Owner decision (2026-10-01, project thread). Amends Q153, R25 (WhatsApp phone OTP and activation) and R26. Business Spec R30.</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs: record R32–R35 in the ledger and close TASK-009/TASK-025
Adds the owner decisions of 2026-10-04 to business-rules-ledger.xlsx
(managed locations, cart merge with its clarification, account
deactivation, cart retention) and marks TASK-009 and TASK-025 Reviewed
and Done, as confirmed by the product owner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/decisions/business-rules-ledger.xlsx
+++ b/docs/decisions/business-rules-ledger.xlsx
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ClosureAuditDecisionsTable" displayName="ClosureAuditDecisionsTable" ref="A1:E30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Decision"/>
@@ -7392,7 +7392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="26" min="1" max="1"/>
@@ -8104,6 +8104,114 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>R32</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Governorates and Areas as a Managed List</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Governorates and their areas form one managed location list shared by customer addresses and shipping rules (Q122); no free text. The 27 Egyptian governorates are preloaded; the Owner/Admin (SHIPPING_MANAGE) adds, renames and deactivates areas. An address names one governorate and one of its areas; deactivated governorates/areas can no longer be chosen, existing addresses keep them.</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-04, TASK-009). Answers TASK-002A open decision 7. Business Spec R32.</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>R33</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Cart Merge After Login</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>When a guest cart is merged into the customer cart, an item present in both gets the sum of the two quantities, capped at the quantity available for that variant; the cap never lowers the quantity already in the customer's own cart (e.g. customer 3, guest 2, 1 available: 3 stays). Items present in only one cart are kept as they are.</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-04, TASK-025); clarification confirmed the same day. API Contract §14, ADR-0031 §4. Business Spec R33.</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>R34</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Customer Account Deactivation</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>The customer deactivates from the profile after entering the current password. Final: signed out everywhere and anonymized immediately (name, email, phone, date of birth, saved addresses). Refused while the customer has an open order, an open return or a non-zero wallet balance. Orders, returns, audit and financial records keep their snapshots. Email and phone are freed for a new account; previous orders are not re-linked.</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-04, TASK-009). Clarifies Q154, Q46. Business Spec R34.</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>R35</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Cart Retention</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>A guest cart expires after 30 days without changes (configurable by the Owner/Admin, setting cart.guest_expiry_days); its token then starts a new empty cart. A customer cart never expires and is kept until checkout. ABANDONED is not used for expiry (left to analytics). Deactivating an account (R34) removes its active cart.</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Owner decision (2026-10-04, TASK-025). ADR-0031. Business Spec R35.</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>